<commit_message>
Add service-grid block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (7):
- blocks/service-grid/service-grid.css
- blocks/service-grid/service-grid.js
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/parsers/service-grid.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","columns","columns","columns"]</t>
+    <t>["hero","service-grid","cards","cards","cards","cards","cards","cards","cards","cards","cards","columns","columns","columns"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-29T05:49:54.640Z</t>
+    <t>2026-04-29T06:19:01.828Z</t>
   </si>
   <si>
     <t>UL Solutions</t>

</xml_diff>

<commit_message>
Add video-text block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (7):
- blocks/video-text/video-text.css
- blocks/video-text/video-text.js
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/parsers/video-text.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero","service-grid","cards","cards","cards","cards","cards","cards","cards","cards","cards","columns","columns","columns"]</t>
+    <t>["hero","service-grid","cards","cards","cards","cards","cards","cards","cards","cards","cards","video-text","columns","columns"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-29T06:19:01.828Z</t>
+    <t>2026-04-29T06:34:10.295Z</t>
   </si>
   <si>
     <t>UL Solutions</t>

</xml_diff>

<commit_message>
Add spotlight-cards block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (7):
- blocks/spotlight-cards/spotlight-cards.css
- blocks/spotlight-cards/spotlight-cards.js
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/parsers/spotlight-cards.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero","service-grid","cards","cards","cards","cards","cards","cards","cards","cards","cards","video-text","columns","columns"]</t>
+    <t>["hero","service-grid","spotlight-cards","cards","cards","cards","cards","cards","cards","cards","cards","video-text","columns","columns"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-29T06:34:10.295Z</t>
+    <t>2026-04-29T06:45:43.072Z</t>
   </si>
   <si>
     <t>UL Solutions</t>

</xml_diff>

<commit_message>
Add feature-cards block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (7):
- blocks/feature-cards/feature-cards.css
- blocks/feature-cards/feature-cards.js
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/parsers/feature-cards.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero","service-grid","spotlight-cards","cards","cards","cards","cards","cards","cards","cards","cards","video-text","columns","columns"]</t>
+    <t>["hero","service-grid","spotlight-cards","feature-cards","cards","cards","cards","cards","cards","cards","cards","video-text","columns","columns"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-29T06:45:43.072Z</t>
+    <t>2026-04-29T06:53:05.900Z</t>
   </si>
   <si>
     <t>UL Solutions</t>

</xml_diff>